<commit_message>
Radio Link coverage map (KML/KMZ/waypoints/pasted coordinates, terrain line of sight); US spelling throughout
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/hangarlab/HangarLab template.xlsx
+++ b/hangarlab/HangarLab template.xlsx
@@ -667,7 +667,7 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Airframes — wingspan, wing area and length in metres, weight in grams.</t>
+          <t>Airframes — wingspan, wing area and length in meters, weight in grams.</t>
         </is>
       </c>
     </row>
@@ -691,7 +691,7 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Units are metric: grams, metres, m², volts, amps, watts, mAh. (The app can still display imperial.)</t>
+          <t>Units are metric: grams, meters, m², volts, amps, watts, mAh. (The app can still display imperial.)</t>
         </is>
       </c>
     </row>
@@ -705,7 +705,7 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>Grey italic rows are examples: overwrite or delete them.</t>
+          <t>Gray italic rows are examples: overwrite or delete them.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
0.3.0-dev: ESC library, ESC and motor limit checks
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/hangarlab/HangarLab template.xlsx
+++ b/hangarlab/HangarLab template.xlsx
@@ -12,9 +12,10 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Motors" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Motor thrust data" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Props" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Batteries" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Airframes" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="8" state="hidden" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ESCs" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Batteries" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Airframes" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="9" state="hidden" r:id="rId9"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -606,7 +607,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A18"/>
+  <dimension ref="A1:A19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
@@ -667,64 +668,71 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Airframes — wingspan, wing area and length in meters, weight in grams.</t>
+          <t>ESCs — continuous and burst current, the cell range it accepts, and weight. Designs pick an ESC for the lift and cruise motors.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
+          <t>Airframes — wingspan, wing area and length in meters, weight in grams.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
           <t>Motor thrust data — thrust-stand tests, one row per measurement: Motor, Prop, Throttle, Thrust, Voltage, Current. Rows with the same Motor + Prop form one test; pick names from the Motors and Props sheets. (Older one-sheet-per-test "Thrust - …" sheets still import.)</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="2" t="inlineStr"/>
-    </row>
     <row r="12">
-      <c r="A12" s="3" t="inlineStr">
+      <c r="A12" s="2" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
         <is>
           <t>Rules</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="2" t="inlineStr">
-        <is>
-          <t>Units are metric: grams, meters, m², volts, amps, watts, mAh. (The app can still display imperial.)</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Keep the header row. Columns can be reordered; extra columns are ignored.</t>
+          <t>Units are metric: grams, meters, m², volts, amps, watts, mAh. (The app can still display imperial.)</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>Gray italic rows are examples: overwrite or delete them.</t>
+          <t>Keep the header row. Columns can be reordered; extra columns are ignored.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Power: Avg W is typical draw, Peak W the worst case. Rail = the supply that powers the part (VBAT = straight from the flight pack).</t>
+          <t>Gray italic rows are examples: overwrite or delete them.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>Link = datasheet or product page. Buy link = where to order it. Unit cost is per item in your currency; the BOM report totals it.</t>
+          <t>Power: Avg W is typical draw, Peak W the worst case. Rail = the supply that powers the part (VBAT = straight from the flight pack).</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>Link = datasheet or product page. Buy link = where to order it. Unit cost is per item in your currency; the BOM report totals it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
         <is>
           <t>Qty in Components is only a reference for your own BOM; the library stores one of each. Add parts to a design in the app.</t>
         </is>
@@ -1999,6 +2007,136 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:J3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="17" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="11" customWidth="1" min="7" max="7"/>
+    <col width="42" customWidth="1" min="8" max="8"/>
+    <col width="11" customWidth="1" min="9" max="9"/>
+    <col width="42" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="22" customHeight="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B1" s="4" t="inlineStr">
+        <is>
+          <t>Brand</t>
+        </is>
+      </c>
+      <c r="C1" s="4" t="inlineStr">
+        <is>
+          <t>Continuous current (A)</t>
+        </is>
+      </c>
+      <c r="D1" s="4" t="inlineStr">
+        <is>
+          <t>Burst current (A)</t>
+        </is>
+      </c>
+      <c r="E1" s="4" t="inlineStr">
+        <is>
+          <t>Min cells (S)</t>
+        </is>
+      </c>
+      <c r="F1" s="4" t="inlineStr">
+        <is>
+          <t>Max cells (S)</t>
+        </is>
+      </c>
+      <c r="G1" s="4" t="inlineStr">
+        <is>
+          <t>Weight (g)</t>
+        </is>
+      </c>
+      <c r="H1" s="4" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
+      <c r="I1" s="4" t="inlineStr">
+        <is>
+          <t>Unit cost</t>
+        </is>
+      </c>
+      <c r="J1" s="4" t="inlineStr">
+        <is>
+          <t>Buy link</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="5" t="inlineStr">
+        <is>
+          <t>Generic 6S 60A ESC</t>
+        </is>
+      </c>
+      <c r="B2" s="5" t="inlineStr"/>
+      <c r="C2" s="5" t="n">
+        <v>60</v>
+      </c>
+      <c r="D2" s="5" t="n">
+        <v>80</v>
+      </c>
+      <c r="E2" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="F2" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="G2" s="5" t="n">
+        <v>60</v>
+      </c>
+      <c r="H2" s="5" t="inlineStr"/>
+      <c r="I2" s="5" t="inlineStr"/>
+      <c r="J2" s="5" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>Generic 12S 80A ESC</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr"/>
+      <c r="C3" s="5" t="n">
+        <v>80</v>
+      </c>
+      <c r="D3" s="5" t="n">
+        <v>100</v>
+      </c>
+      <c r="E3" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="F3" s="5" t="n">
+        <v>12</v>
+      </c>
+      <c r="G3" s="5" t="n">
+        <v>90</v>
+      </c>
+      <c r="H3" s="5" t="inlineStr"/>
+      <c r="I3" s="5" t="inlineStr"/>
+      <c r="J3" s="5" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:K3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -2156,7 +2294,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2274,7 +2412,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
0.5.0-dev: ESC For column (multirotor / plane / either)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/hangarlab/HangarLab template.xlsx
+++ b/hangarlab/HangarLab template.xlsx
@@ -2007,19 +2007,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J3"/>
+  <dimension ref="A1:K3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
-    <col width="17" customWidth="1" min="4" max="4"/>
-    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="17" customWidth="1" min="5" max="5"/>
     <col width="13" customWidth="1" min="6" max="6"/>
-    <col width="11" customWidth="1" min="7" max="7"/>
-    <col width="42" customWidth="1" min="8" max="8"/>
-    <col width="11" customWidth="1" min="9" max="9"/>
-    <col width="42" customWidth="1" min="10" max="10"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="11" customWidth="1" min="8" max="8"/>
+    <col width="42" customWidth="1" min="9" max="9"/>
+    <col width="11" customWidth="1" min="10" max="10"/>
+    <col width="42" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
@@ -2035,40 +2036,45 @@
       </c>
       <c r="C1" s="4" t="inlineStr">
         <is>
+          <t>For (Multirotor / Plane / Either)</t>
+        </is>
+      </c>
+      <c r="D1" s="4" t="inlineStr">
+        <is>
           <t>Continuous current (A)</t>
         </is>
       </c>
-      <c r="D1" s="4" t="inlineStr">
+      <c r="E1" s="4" t="inlineStr">
         <is>
           <t>Burst current (A)</t>
         </is>
       </c>
-      <c r="E1" s="4" t="inlineStr">
+      <c r="F1" s="4" t="inlineStr">
         <is>
           <t>Min cells (S)</t>
         </is>
       </c>
-      <c r="F1" s="4" t="inlineStr">
+      <c r="G1" s="4" t="inlineStr">
         <is>
           <t>Max cells (S)</t>
         </is>
       </c>
-      <c r="G1" s="4" t="inlineStr">
+      <c r="H1" s="4" t="inlineStr">
         <is>
           <t>Weight (g)</t>
         </is>
       </c>
-      <c r="H1" s="4" t="inlineStr">
+      <c r="I1" s="4" t="inlineStr">
         <is>
           <t>Link</t>
         </is>
       </c>
-      <c r="I1" s="4" t="inlineStr">
+      <c r="J1" s="4" t="inlineStr">
         <is>
           <t>Unit cost</t>
         </is>
       </c>
-      <c r="J1" s="4" t="inlineStr">
+      <c r="K1" s="4" t="inlineStr">
         <is>
           <t>Buy link</t>
         </is>
@@ -2081,24 +2087,29 @@
         </is>
       </c>
       <c r="B2" s="5" t="inlineStr"/>
-      <c r="C2" s="5" t="n">
+      <c r="C2" s="5" t="inlineStr">
+        <is>
+          <t>Either</t>
+        </is>
+      </c>
+      <c r="D2" s="5" t="n">
         <v>60</v>
       </c>
-      <c r="D2" s="5" t="n">
+      <c r="E2" s="5" t="n">
         <v>80</v>
       </c>
-      <c r="E2" s="5" t="n">
+      <c r="F2" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="F2" s="5" t="n">
+      <c r="G2" s="5" t="n">
         <v>6</v>
       </c>
-      <c r="G2" s="5" t="n">
+      <c r="H2" s="5" t="n">
         <v>60</v>
       </c>
-      <c r="H2" s="5" t="inlineStr"/>
       <c r="I2" s="5" t="inlineStr"/>
       <c r="J2" s="5" t="inlineStr"/>
+      <c r="K2" s="5" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
@@ -2107,24 +2118,29 @@
         </is>
       </c>
       <c r="B3" s="5" t="inlineStr"/>
-      <c r="C3" s="5" t="n">
+      <c r="C3" s="5" t="inlineStr">
+        <is>
+          <t>Multirotor</t>
+        </is>
+      </c>
+      <c r="D3" s="5" t="n">
         <v>80</v>
       </c>
-      <c r="D3" s="5" t="n">
+      <c r="E3" s="5" t="n">
         <v>100</v>
       </c>
-      <c r="E3" s="5" t="n">
+      <c r="F3" s="5" t="n">
         <v>6</v>
       </c>
-      <c r="F3" s="5" t="n">
+      <c r="G3" s="5" t="n">
         <v>12</v>
       </c>
-      <c r="G3" s="5" t="n">
+      <c r="H3" s="5" t="n">
         <v>90</v>
       </c>
-      <c r="H3" s="5" t="inlineStr"/>
       <c r="I3" s="5" t="inlineStr"/>
       <c r="J3" s="5" t="inlineStr"/>
+      <c r="K3" s="5" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
0.6.0-dev: multirotor frames, airframe types, prop clearance check
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/hangarlab/HangarLab template.xlsx
+++ b/hangarlab/HangarLab template.xlsx
@@ -675,7 +675,7 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Airframes — wingspan, wing area and length in meters, weight in grams.</t>
+          <t>Airframes — type, then wingspan, wing area and length in meters for wings, or wheelbase (mm), layout and max prop size for multirotor frames; weight in grams.</t>
         </is>
       </c>
     </row>
@@ -2316,18 +2316,22 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I3"/>
+  <dimension ref="A1:M4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="15" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="30" customWidth="1" min="6" max="6"/>
-    <col width="42" customWidth="1" min="7" max="7"/>
-    <col width="11" customWidth="1" min="8" max="8"/>
-    <col width="42" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="30" customWidth="1" min="10" max="10"/>
+    <col width="42" customWidth="1" min="11" max="11"/>
+    <col width="11" customWidth="1" min="12" max="12"/>
+    <col width="42" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
@@ -2338,40 +2342,60 @@
       </c>
       <c r="B1" s="4" t="inlineStr">
         <is>
+          <t>Type (Fixed-wing / Multirotor / Hybrid VTOL)</t>
+        </is>
+      </c>
+      <c r="C1" s="4" t="inlineStr">
+        <is>
           <t>Wingspan (m)</t>
         </is>
       </c>
-      <c r="C1" s="4" t="inlineStr">
+      <c r="D1" s="4" t="inlineStr">
         <is>
           <t>Wing area (m²)</t>
         </is>
       </c>
-      <c r="D1" s="4" t="inlineStr">
+      <c r="E1" s="4" t="inlineStr">
         <is>
           <t>Length (m)</t>
         </is>
       </c>
-      <c r="E1" s="4" t="inlineStr">
+      <c r="F1" s="4" t="inlineStr">
+        <is>
+          <t>Wheelbase (mm)</t>
+        </is>
+      </c>
+      <c r="G1" s="4" t="inlineStr">
+        <is>
+          <t>Layout (Quad X, Hexa, ...)</t>
+        </is>
+      </c>
+      <c r="H1" s="4" t="inlineStr">
+        <is>
+          <t>Max prop (in)</t>
+        </is>
+      </c>
+      <c r="I1" s="4" t="inlineStr">
         <is>
           <t>Weight (g)</t>
         </is>
       </c>
-      <c r="F1" s="4" t="inlineStr">
+      <c r="J1" s="4" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
-      <c r="G1" s="4" t="inlineStr">
+      <c r="K1" s="4" t="inlineStr">
         <is>
           <t>Link</t>
         </is>
       </c>
-      <c r="H1" s="4" t="inlineStr">
+      <c r="L1" s="4" t="inlineStr">
         <is>
           <t>Unit cost</t>
         </is>
       </c>
-      <c r="I1" s="4" t="inlineStr">
+      <c r="M1" s="4" t="inlineStr">
         <is>
           <t>Buy link</t>
         </is>
@@ -2383,22 +2407,30 @@
           <t>AtomRC Dolphin Pro</t>
         </is>
       </c>
-      <c r="B2" s="5" t="n">
+      <c r="B2" s="5" t="inlineStr">
+        <is>
+          <t>Fixed-wing</t>
+        </is>
+      </c>
+      <c r="C2" s="5" t="n">
         <v>0.845</v>
       </c>
-      <c r="C2" s="5" t="n">
+      <c r="D2" s="5" t="n">
         <v>0.1696</v>
       </c>
-      <c r="D2" s="5" t="n">
+      <c r="E2" s="5" t="n">
         <v>0.826</v>
-      </c>
-      <c r="E2" s="5" t="n">
-        <v>790</v>
       </c>
       <c r="F2" s="5" t="inlineStr"/>
       <c r="G2" s="5" t="inlineStr"/>
       <c r="H2" s="5" t="inlineStr"/>
-      <c r="I2" s="5" t="inlineStr"/>
+      <c r="I2" s="5" t="n">
+        <v>790</v>
+      </c>
+      <c r="J2" s="5" t="inlineStr"/>
+      <c r="K2" s="5" t="inlineStr"/>
+      <c r="L2" s="5" t="inlineStr"/>
+      <c r="M2" s="5" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
@@ -2406,22 +2438,67 @@
           <t>HEEWING T2 Cruza</t>
         </is>
       </c>
-      <c r="B3" s="5" t="n">
+      <c r="B3" s="5" t="inlineStr">
+        <is>
+          <t>Fixed-wing</t>
+        </is>
+      </c>
+      <c r="C3" s="5" t="n">
         <v>1.2</v>
       </c>
-      <c r="C3" s="5" t="inlineStr"/>
       <c r="D3" s="5" t="inlineStr"/>
-      <c r="E3" s="5" t="n">
-        <v>1200</v>
-      </c>
-      <c r="F3" s="5" t="inlineStr">
-        <is>
-          <t>wing area not listed</t>
-        </is>
-      </c>
+      <c r="E3" s="5" t="inlineStr"/>
+      <c r="F3" s="5" t="inlineStr"/>
       <c r="G3" s="5" t="inlineStr"/>
       <c r="H3" s="5" t="inlineStr"/>
-      <c r="I3" s="5" t="inlineStr"/>
+      <c r="I3" s="5" t="n">
+        <v>1200</v>
+      </c>
+      <c r="J3" s="5" t="inlineStr">
+        <is>
+          <t>wing area not listed</t>
+        </is>
+      </c>
+      <c r="K3" s="5" t="inlineStr"/>
+      <c r="L3" s="5" t="inlineStr"/>
+      <c r="M3" s="5" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>Example 500 mm quad frame</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>Multirotor</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr"/>
+      <c r="D4" s="5" t="inlineStr"/>
+      <c r="E4" s="5" t="inlineStr"/>
+      <c r="F4" s="5" t="n">
+        <v>500</v>
+      </c>
+      <c r="G4" s="5" t="inlineStr">
+        <is>
+          <t>Quad X</t>
+        </is>
+      </c>
+      <c r="H4" s="5" t="n">
+        <v>13</v>
+      </c>
+      <c r="I4" s="5" t="n">
+        <v>450</v>
+      </c>
+      <c r="J4" s="5" t="inlineStr">
+        <is>
+          <t>multirotor: wheelbase, layout and max prop instead of a wing</t>
+        </is>
+      </c>
+      <c r="K4" s="5" t="inlineStr"/>
+      <c r="L4" s="5" t="inlineStr"/>
+      <c r="M4" s="5" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>